<commit_message>
Updated template and processing
</commit_message>
<xml_diff>
--- a/data/utils/excel_template_v0.01.xlsx
+++ b/data/utils/excel_template_v0.01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mkerri\Documents\My Projects\2. In Progress\Auxiliary\10. Traffic Regression Tool\Traffic-Regression-Tool\data\utils\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC115C96-7FE1-4F8C-97BC-196E55D78D24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2158836F-B2E1-42BF-93DA-92E03D8FFC3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BasicSheet" sheetId="4" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t>END</t>
   </si>
@@ -51,6 +51,63 @@
   </si>
   <si>
     <t>[Insert heading here]</t>
+  </si>
+  <si>
+    <t>Excel Template Instructions:</t>
+  </si>
+  <si>
+    <t>1.  **Single Sheet Only:** Use ONLY the first sheet.</t>
+  </si>
+  <si>
+    <t>2.  **Variable Names (Column D):**</t>
+  </si>
+  <si>
+    <t>*   List all variable names in Column D.</t>
+  </si>
+  <si>
+    <t>*   Place under "Dependent Variables" or "Independent Variables" headers (do not change these header texts).</t>
+  </si>
+  <si>
+    <t>3.  **Variable Types (Column E):**</t>
+  </si>
+  <si>
+    <t>4.  **Data Values (Column G onwards):**</t>
+  </si>
+  <si>
+    <t>*   Enter numerical data for each variable starting in Column G.</t>
+  </si>
+  <si>
+    <t>*   No empty cells or text within the data range for a variable.</t>
+  </si>
+  <si>
+    <t>5.  **Timeline:**</t>
+  </si>
+  <si>
+    <t>6.  **Seasonality Variables:**</t>
+  </si>
+  <si>
+    <t>*   Best added via the app's "Input Template" page.</t>
+  </si>
+  <si>
+    <t>*   Do not use "Seasonality" in names of non-seasonality variables.</t>
+  </si>
+  <si>
+    <t>*   For each variable in Col D, specify its type in Col E as "value" or "dummy".</t>
+  </si>
+  <si>
+    <t>*   If adding manually, ensure they are added as "dummy" type.</t>
+  </si>
+  <si>
+    <t>*   Ensure all variable names are unique. Do not add any other info to Column D.</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>*   Do not add any other info to Column E.</t>
+  </si>
+  <si>
+    <t>*   The data timeline is defined by the headers in Row 33 (starting Col G).</t>
   </si>
 </sst>
 </file>
@@ -686,7 +743,7 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1">
       <alignment vertical="center"/>
@@ -699,6 +756,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="33" applyNumberFormat="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="7">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="54">
@@ -1071,14 +1131,14 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:S40"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="B2:S60"/>
+  <sheetFormatPr defaultColWidth="9.09765625" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="19" width="9.140625" customWidth="1"/>
+    <col min="2" max="19" width="9.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:19" ht="17.25" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:19" ht="17" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
@@ -1100,7 +1160,7 @@
       <c r="R2" s="1"/>
       <c r="S2" s="1"/>
     </row>
-    <row r="3" spans="2:19" ht="17.25" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:19" ht="17" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1122,7 +1182,7 @@
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
     </row>
-    <row r="4" spans="2:19" ht="17.25" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:19" ht="17" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1144,7 +1204,7 @@
       <c r="R4" s="1"/>
       <c r="S4" s="1"/>
     </row>
-    <row r="6" spans="2:19" ht="17.25" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:19" ht="17" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
@@ -1166,36 +1226,170 @@
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
     </row>
-    <row r="12" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="D12" s="4"/>
-    </row>
-    <row r="13" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="D13" s="2"/>
-    </row>
-    <row r="14" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="D14" s="3"/>
-    </row>
-    <row r="40" spans="2:19" ht="17.25" x14ac:dyDescent="0.2">
-      <c r="B40" s="1" t="s">
+    <row r="8" spans="2:19" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="B8" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
+      <c r="O8" s="5"/>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="5"/>
+      <c r="R8" s="5"/>
+      <c r="S8" s="5"/>
+    </row>
+    <row r="10" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="C13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="C14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="C16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="C17" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B18" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="C19" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="C20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B21" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="C22" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="C23" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="C25" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="C26" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="27" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="C27" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="2:19" ht="15.5" x14ac:dyDescent="0.3">
+      <c r="B29" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="5"/>
+      <c r="O29" s="5"/>
+      <c r="P29" s="5"/>
+      <c r="Q29" s="5"/>
+      <c r="R29" s="5"/>
+      <c r="S29" s="5"/>
+    </row>
+    <row r="32" spans="2:19" x14ac:dyDescent="0.3">
+      <c r="D32" s="4"/>
+    </row>
+    <row r="33" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D33" s="2"/>
+    </row>
+    <row r="34" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D34" s="3"/>
+    </row>
+    <row r="60" spans="2:19" ht="17" x14ac:dyDescent="0.3">
+      <c r="B60" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C40" s="1"/>
-      <c r="D40" s="1"/>
-      <c r="E40" s="1"/>
-      <c r="F40" s="1"/>
-      <c r="G40" s="1"/>
-      <c r="H40" s="1"/>
-      <c r="I40" s="1"/>
-      <c r="J40" s="1"/>
-      <c r="K40" s="1"/>
-      <c r="L40" s="1"/>
-      <c r="M40" s="1"/>
-      <c r="N40" s="1"/>
-      <c r="O40" s="1"/>
-      <c r="P40" s="1"/>
-      <c r="Q40" s="1"/>
-      <c r="R40" s="1"/>
-      <c r="S40" s="1"/>
+      <c r="C60" s="1"/>
+      <c r="D60" s="1"/>
+      <c r="E60" s="1"/>
+      <c r="F60" s="1"/>
+      <c r="G60" s="1"/>
+      <c r="H60" s="1"/>
+      <c r="I60" s="1"/>
+      <c r="J60" s="1"/>
+      <c r="K60" s="1"/>
+      <c r="L60" s="1"/>
+      <c r="M60" s="1"/>
+      <c r="N60" s="1"/>
+      <c r="O60" s="1"/>
+      <c r="P60" s="1"/>
+      <c r="Q60" s="1"/>
+      <c r="R60" s="1"/>
+      <c r="S60" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>